<commit_message>
feat: Public Profile Page and test
</commit_message>
<xml_diff>
--- a/resources/UserDetails.xlsx
+++ b/resources/UserDetails.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Email</t>
   </si>
@@ -27,6 +27,21 @@
   </si>
   <si>
     <t>MsKurtisJenkins@yopmail.com</t>
+  </si>
+  <si>
+    <t>MonaBlock@yopmail.com</t>
+  </si>
+  <si>
+    <t>MrsSonLeannon@yopmail.com</t>
+  </si>
+  <si>
+    <t>DrJoesphStoltenberg@yopmail.com</t>
+  </si>
+  <si>
+    <t>MrsJeffersonToy@yopmail.com</t>
+  </si>
+  <si>
+    <t>TylerPadberg@yopmail.com</t>
   </si>
 </sst>
 </file>
@@ -71,7 +86,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -99,6 +114,31 @@
         <v>4</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Browser Issue Resolved in Public Profile
</commit_message>
<xml_diff>
--- a/resources/UserDetails.xlsx
+++ b/resources/UserDetails.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Email</t>
   </si>
@@ -42,6 +42,15 @@
   </si>
   <si>
     <t>TylerPadberg@yopmail.com</t>
+  </si>
+  <si>
+    <t>AdolfoConnelly@yopmail.com</t>
+  </si>
+  <si>
+    <t>ClydeBernier@yopmail.com</t>
+  </si>
+  <si>
+    <t>BobetteKreiger@yopmail.com</t>
   </si>
 </sst>
 </file>
@@ -86,7 +95,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -139,6 +148,21 @@
         <v>9</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>12</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: updated resources, suite and testng xml files
</commit_message>
<xml_diff>
--- a/resources/UserDetails.xlsx
+++ b/resources/UserDetails.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
   <si>
     <t>Email</t>
   </si>
@@ -53,10 +53,13 @@
     <t>BobetteKreiger@yopmail.com</t>
   </si>
   <si>
-    <t>AdamZulauf@yopmail.com</t>
-  </si>
-  <si>
-    <t>AlejandroPriceDVM@yopmail.com</t>
+    <t>BusterGerhold@yopmail.com</t>
+  </si>
+  <si>
+    <t>BasilDonnelly@yopmail.com</t>
+  </si>
+  <si>
+    <t>IrwinGreenfelder@yopmail.com</t>
   </si>
 </sst>
 </file>
@@ -101,7 +104,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -189,6 +192,11 @@
         <v>14</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="s" s="0">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>